<commit_message>
Implemented Excel-driven DataProvider framework with Apache POI integration, resolved sheet lookup NullPointerException, and validated multi-dataset TestNG execution
</commit_message>
<xml_diff>
--- a/testdata/LoginData.xlsx
+++ b/testdata/LoginData.xlsx
@@ -5,15 +5,15 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vishw\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vishw\eclipse-workspace\E2EHybridFramework\saucedemohybridframework\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{22A4FF3E-3906-489B-A834-624C216B0588}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{75FDD6EE-19B1-4696-A9D6-E5A1279604EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C1196554-70E1-419D-81E4-3025B88BF07D}"/>
+    <workbookView xWindow="2268" yWindow="2268" windowWidth="17280" windowHeight="8880" xr2:uid="{C1196554-70E1-419D-81E4-3025B88BF07D}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="LoginData" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>